<commit_message>
test(TC_FUNC_01): Reject an incorrect password for a known username
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -503,21 +503,14 @@
       <x:c r="N2" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O2" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P2" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q2" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O2" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P2" s="2" t="str">
+        <x:v>1. Nhập username + invalid_password; bấm Đăng nhập; chờ phản hồi.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công.</x:v>
+      </x:c>
+      <x:c r="Q2" s="2" t="str"/>
       <x:c r="R2" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -2953,26 +2946,17 @@
       <x:c r="A2" s="2" t="str">
         <x:v>TC_FUNC_01</x:v>
       </x:c>
-      <x:c r="B2" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D2" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E2" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B2" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C2" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_FUNC_01</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="str">
+        <x:v>1. Nhập username + invalid_password; bấm Đăng nhập; chờ phản hồi.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công.</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="str"/>
     </x:row>
     <x:row r="3" ht="108.75" customHeight="1">
       <x:c r="A3" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_FUNC_02): Reject a blank username
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -557,21 +557,14 @@
       <x:c r="N3" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O3" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P3" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q3" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O3" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P3" s="2" t="str">
+        <x:v>1. Bỏ trống username, điền password sai, submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Có validation native kèm message hoặc thông báo lỗi server; form login còn hiển thị.</x:v>
+      </x:c>
+      <x:c r="Q3" s="2" t="str"/>
       <x:c r="R3" s="2" t="str">
         <x:v>{"empty_field":"username","auth_flow":true,"error_text":"Bạn chưa nhập tên đăng nhập"}</x:v>
       </x:c>
@@ -2962,26 +2955,17 @@
       <x:c r="A3" s="2" t="str">
         <x:v>TC_FUNC_02</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D3" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E3" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B3" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_FUNC_02</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="str">
+        <x:v>1. Bỏ trống username, điền password sai, submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Có validation native kèm message hoặc thông báo lỗi server; form login còn hiển thị.</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="str"/>
     </x:row>
     <x:row r="4" ht="108.75" customHeight="1">
       <x:c r="A4" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_FUNC_03): Reject a blank password
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -611,21 +611,14 @@
       <x:c r="N4" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O4" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P4" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q4" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O4" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P4" s="2" t="str">
+        <x:v>1. Điền username, bỏ password, submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Có validation native kèm message hoặc thông báo lỗi server; form login còn hiển thị.</x:v>
+      </x:c>
+      <x:c r="Q4" s="2" t="str"/>
       <x:c r="R4" s="2" t="str">
         <x:v>{"empty_field":"password","auth_flow":true,"error_text":"Bạn chưa nhập mật khẩu"}</x:v>
       </x:c>
@@ -2971,26 +2964,17 @@
       <x:c r="A4" s="2" t="str">
         <x:v>TC_FUNC_03</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D4" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B4" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_FUNC_03</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="str">
+        <x:v>1. Điền username, bỏ password, submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Có validation native kèm message hoặc thông báo lỗi server; form login còn hiển thị.</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="str"/>
     </x:row>
     <x:row r="5" ht="108.75" customHeight="1">
       <x:c r="A5" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_FUNC_04): Reject blank username and password
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -665,21 +665,14 @@
       <x:c r="N5" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O5" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P5" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q5" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O5" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P5" s="2" t="str">
+        <x:v>1. Bỏ trống hai trường rồi submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Có validation native kèm message hoặc thông báo lỗi server; form login còn hiển thị.</x:v>
+      </x:c>
+      <x:c r="Q5" s="2" t="str"/>
       <x:c r="R5" s="2" t="str">
         <x:v>{"empty_field":"both","auth_flow":true,"error_text":"Bạn chưa nhập tên đăng nhập"}</x:v>
       </x:c>
@@ -2980,26 +2973,17 @@
       <x:c r="A5" s="2" t="str">
         <x:v>TC_FUNC_04</x:v>
       </x:c>
-      <x:c r="B5" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D5" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E5" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B5" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C5" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_FUNC_04</x:v>
+      </x:c>
+      <x:c r="D5" s="2" t="str">
+        <x:v>1. Bỏ trống hai trường rồi submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Có validation native kèm message hoặc thông báo lỗi server; form login còn hiển thị.</x:v>
+      </x:c>
+      <x:c r="E5" s="2" t="str"/>
     </x:row>
     <x:row r="6" ht="108.75" customHeight="1">
       <x:c r="A6" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_FUNC_05): Reject a nonexistent username
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -719,21 +719,14 @@
       <x:c r="N6" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O6" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P6" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q6" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O6" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P6" s="2" t="str">
+        <x:v>1. Nhập username không tồn tại + mật khẩu sai rồi submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công.</x:v>
+      </x:c>
+      <x:c r="Q6" s="2" t="str"/>
       <x:c r="R6" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -2989,26 +2982,17 @@
       <x:c r="A6" s="2" t="str">
         <x:v>TC_FUNC_05</x:v>
       </x:c>
-      <x:c r="B6" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D6" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E6" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B6" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_FUNC_05</x:v>
+      </x:c>
+      <x:c r="D6" s="2" t="str">
+        <x:v>1. Nhập username không tồn tại + mật khẩu sai rồi submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công.</x:v>
+      </x:c>
+      <x:c r="E6" s="2" t="str"/>
     </x:row>
     <x:row r="7" ht="108.75" customHeight="1">
       <x:c r="A7" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_FUNC_06): Reject credentials when username and password are swapped
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -773,21 +773,14 @@
       <x:c r="N7" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O7" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P7" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q7" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O7" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P7" s="2" t="str">
+        <x:v>1. Nhập hai giá trị sai hoán đổi vị trí, submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công.</x:v>
+      </x:c>
+      <x:c r="Q7" s="2" t="str"/>
       <x:c r="R7" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -2998,26 +2991,17 @@
       <x:c r="A7" s="2" t="str">
         <x:v>TC_FUNC_06</x:v>
       </x:c>
-      <x:c r="B7" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C7" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D7" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E7" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B7" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_FUNC_06</x:v>
+      </x:c>
+      <x:c r="D7" s="2" t="str">
+        <x:v>1. Nhập hai giá trị sai hoán đổi vị trí, submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công.</x:v>
+      </x:c>
+      <x:c r="E7" s="2" t="str"/>
     </x:row>
     <x:row r="8" ht="108.75" customHeight="1">
       <x:c r="A8" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_FUNC_07): Reject a case-altered password
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -827,21 +827,14 @@
       <x:c r="N8" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O8" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P8" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q8" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O8" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P8" s="2" t="str">
+        <x:v>1. Đổi hoa/thường chuỗi password sai đã biết, submit với username cấu hình.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không suy ra tính phân biệt của mật khẩu hợp lệ.</x:v>
+      </x:c>
+      <x:c r="Q8" s="2" t="str"/>
       <x:c r="R8" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3007,26 +3000,17 @@
       <x:c r="A8" s="2" t="str">
         <x:v>TC_FUNC_07</x:v>
       </x:c>
-      <x:c r="B8" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C8" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D8" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E8" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B8" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C8" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_FUNC_07</x:v>
+      </x:c>
+      <x:c r="D8" s="2" t="str">
+        <x:v>1. Đổi hoa/thường chuỗi password sai đã biết, submit với username cấu hình.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không suy ra tính phân biệt của mật khẩu hợp lệ.</x:v>
+      </x:c>
+      <x:c r="E8" s="2" t="str"/>
     </x:row>
     <x:row r="9" ht="108.75" customHeight="1">
       <x:c r="A9" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_FUNC_08): Reject invalid credentials with Remember Me selected
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -881,21 +881,14 @@
       <x:c r="N9" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O9" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P9" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q9" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O9" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P9" s="2" t="str">
+        <x:v>1. Chọn checkbox nếu chưa chọn; kiểm tra selected=true; submit dữ liệu sai.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Trạng thái checkbox được kiểm tra trước submit; không kiểm tra persistence.</x:v>
+      </x:c>
+      <x:c r="Q9" s="2" t="str"/>
       <x:c r="R9" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3016,26 +3009,17 @@
       <x:c r="A9" s="2" t="str">
         <x:v>TC_FUNC_08</x:v>
       </x:c>
-      <x:c r="B9" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C9" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D9" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E9" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B9" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C9" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_FUNC_08</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="str">
+        <x:v>1. Chọn checkbox nếu chưa chọn; kiểm tra selected=true; submit dữ liệu sai.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Trạng thái checkbox được kiểm tra trước submit; không kiểm tra persistence.</x:v>
+      </x:c>
+      <x:c r="E9" s="2" t="str"/>
     </x:row>
     <x:row r="10" ht="108.75" customHeight="1">
       <x:c r="A10" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_FUNC_09): Reject invalid credentials with Remember Me cleared
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -935,21 +935,14 @@
       <x:c r="N10" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O10" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P10" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q10" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O10" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P10" s="2" t="str">
+        <x:v>1. Bỏ chọn nếu đang chọn; kiểm tra selected=false; submit dữ liệu sai.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không kiểm tra cookie persistence.</x:v>
+      </x:c>
+      <x:c r="Q10" s="2" t="str"/>
       <x:c r="R10" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3025,26 +3018,17 @@
       <x:c r="A10" s="2" t="str">
         <x:v>TC_FUNC_09</x:v>
       </x:c>
-      <x:c r="B10" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C10" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D10" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E10" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B10" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_FUNC_09</x:v>
+      </x:c>
+      <x:c r="D10" s="2" t="str">
+        <x:v>1. Bỏ chọn nếu đang chọn; kiểm tra selected=false; submit dữ liệu sai.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không kiểm tra cookie persistence.</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="str"/>
     </x:row>
     <x:row r="11" ht="108.75" customHeight="1">
       <x:c r="A11" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_FUNC_10): Reject invalid credentials submitted with Enter
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -989,21 +989,14 @@
       <x:c r="N11" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O11" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P11" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q11" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O11" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P11" s="2" t="str">
+        <x:v>1. Nhập dữ liệu sai; nhấn Enter tại password; chờ thông báo.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công.</x:v>
+      </x:c>
+      <x:c r="Q11" s="2" t="str"/>
       <x:c r="R11" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3034,26 +3027,17 @@
       <x:c r="A11" s="2" t="str">
         <x:v>TC_FUNC_10</x:v>
       </x:c>
-      <x:c r="B11" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C11" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D11" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E11" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B11" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C11" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_FUNC_10</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="str">
+        <x:v>1. Nhập dữ liệu sai; nhấn Enter tại password; chờ thông báo.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công.</x:v>
+      </x:c>
+      <x:c r="E11" s="2" t="str"/>
     </x:row>
     <x:row r="12" ht="108.75" customHeight="1">
       <x:c r="A12" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_FUNC_11): Show the login page when opened without a session
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1043,21 +1043,14 @@
       <x:c r="N12" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O12" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P12" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q12" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O12" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P12" s="2" t="str">
+        <x:v>1. Truy cập URL auth không có credentials.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Username/password/nút login hiển thị. Không suy ra authorization của URL nội bộ.</x:v>
+      </x:c>
+      <x:c r="Q12" s="2" t="str"/>
       <x:c r="R12" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3043,26 +3036,17 @@
       <x:c r="A12" s="2" t="str">
         <x:v>TC_FUNC_11</x:v>
       </x:c>
-      <x:c r="B12" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D12" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E12" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B12" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_FUNC_11</x:v>
+      </x:c>
+      <x:c r="D12" s="2" t="str">
+        <x:v>1. Truy cập URL auth không có credentials.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Username/password/nút login hiển thị. Không suy ra authorization của URL nội bộ.</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="str"/>
     </x:row>
     <x:row r="13" ht="108.75" customHeight="1">
       <x:c r="A13" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_FUNC_12): Keep the login page after refreshing a failed authentication
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1097,21 +1097,14 @@
       <x:c r="N13" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O13" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P13" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q13" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O13" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P13" s="2" t="str">
+        <x:v>1. Submit sai, xác nhận lỗi, refresh trang.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Sau refresh form login vẫn hiển thị; không yêu cầu phiên đã xác thực.</x:v>
+      </x:c>
+      <x:c r="Q13" s="2" t="str"/>
       <x:c r="R13" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3052,26 +3045,17 @@
       <x:c r="A13" s="2" t="str">
         <x:v>TC_FUNC_12</x:v>
       </x:c>
-      <x:c r="B13" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C13" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D13" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E13" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B13" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_FUNC_12</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="str">
+        <x:v>1. Submit sai, xác nhận lỗi, refresh trang.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Sau refresh form login vẫn hiển thị; không yêu cầu phiên đã xác thực.</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="str"/>
     </x:row>
     <x:row r="14" ht="108.75" customHeight="1">
       <x:c r="A14" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_BND_01): Reject a username with leading and trailing whitespace
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1151,21 +1151,14 @@
       <x:c r="N14" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O14" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P14" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q14" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O14" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P14" s="2" t="str">
+        <x:v>1. Nhập dữ liệu có space đầu/cuối và submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không suy ra chính sách trim của username hợp lệ.</x:v>
+      </x:c>
+      <x:c r="Q14" s="2" t="str"/>
       <x:c r="R14" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3061,26 +3054,17 @@
       <x:c r="A14" s="2" t="str">
         <x:v>TC_BND_01</x:v>
       </x:c>
-      <x:c r="B14" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C14" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D14" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E14" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B14" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_BND_01</x:v>
+      </x:c>
+      <x:c r="D14" s="2" t="str">
+        <x:v>1. Nhập dữ liệu có space đầu/cuối và submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không suy ra chính sách trim của username hợp lệ.</x:v>
+      </x:c>
+      <x:c r="E14" s="2" t="str"/>
     </x:row>
     <x:row r="15" ht="108.75" customHeight="1">
       <x:c r="A15" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_BND_02): Reject a username with embedded whitespace
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1205,21 +1205,14 @@
       <x:c r="N15" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O15" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P15" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q15" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O15" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P15" s="2" t="str">
+        <x:v>1. Nhập username có space ở giữa và submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công.</x:v>
+      </x:c>
+      <x:c r="Q15" s="2" t="str"/>
       <x:c r="R15" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3070,26 +3063,17 @@
       <x:c r="A15" s="2" t="str">
         <x:v>TC_BND_02</x:v>
       </x:c>
-      <x:c r="B15" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C15" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D15" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E15" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B15" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_BND_02</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="str">
+        <x:v>1. Nhập username có space ở giữa và submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công.</x:v>
+      </x:c>
+      <x:c r="E15" s="2" t="str"/>
     </x:row>
     <x:row r="16" ht="108.75" customHeight="1">
       <x:c r="A16" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_BND_03): Reject invalid usernames at lengths 1, 255, and 256
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1259,21 +1259,14 @@
       <x:c r="N16" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O16" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P16" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q16" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O16" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P16" s="2" t="str">
+        <x:v>1. Mỗi mẫu: phiên chưa login; nhập username dài và password sai; submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Đây là xử lý dữ liệu dài, không xác nhận maxlength chính sách.</x:v>
+      </x:c>
+      <x:c r="Q16" s="2" t="str"/>
       <x:c r="R16" s="2" t="str">
         <x:v>{"lengths":[1,255,256],"auth_flow":true}</x:v>
       </x:c>
@@ -3079,26 +3072,17 @@
       <x:c r="A16" s="2" t="str">
         <x:v>TC_BND_03</x:v>
       </x:c>
-      <x:c r="B16" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C16" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D16" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E16" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B16" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_BND_03</x:v>
+      </x:c>
+      <x:c r="D16" s="2" t="str">
+        <x:v>1. Mỗi mẫu: phiên chưa login; nhập username dài và password sai; submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Đây là xử lý dữ liệu dài, không xác nhận maxlength chính sách.</x:v>
+      </x:c>
+      <x:c r="E16" s="2" t="str"/>
     </x:row>
     <x:row r="17" ht="108.75" customHeight="1">
       <x:c r="A17" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_BND_04): Reject invalid passwords at lengths 1, 255, and 256
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1313,21 +1313,14 @@
       <x:c r="N17" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O17" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P17" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q17" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O17" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P17" s="2" t="str">
+        <x:v>1. Mỗi mẫu: nhập username không tồn tại và password dài; submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không suy ra thuật toán hash hoặc maxlength chính sách.</x:v>
+      </x:c>
+      <x:c r="Q17" s="2" t="str"/>
       <x:c r="R17" s="2" t="str">
         <x:v>{"lengths":[1,255,256],"auth_flow":true}</x:v>
       </x:c>
@@ -3088,26 +3081,17 @@
       <x:c r="A17" s="2" t="str">
         <x:v>TC_BND_04</x:v>
       </x:c>
-      <x:c r="B17" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C17" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D17" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E17" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B17" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_BND_04</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="str">
+        <x:v>1. Mỗi mẫu: nhập username không tồn tại và password dài; submit.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không suy ra thuật toán hash hoặc maxlength chính sách.</x:v>
+      </x:c>
+      <x:c r="E17" s="2" t="str"/>
     </x:row>
     <x:row r="18" ht="108.75" customHeight="1">
       <x:c r="A18" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_BND_05): Reject invalid Unicode credentials
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1367,21 +1367,14 @@
       <x:c r="N18" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O18" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P18" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q18" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O18" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P18" s="2" t="str">
+        <x:v>1. Nhập hai chuỗi Unicode sai, submit; kiểm tra HTML không có ký tự thay thế U+FFFD.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không suy ra hỗ trợ tài khoản Unicode hợp lệ.</x:v>
+      </x:c>
+      <x:c r="Q18" s="2" t="str"/>
       <x:c r="R18" s="2" t="str">
         <x:v>{"username":"tài_khoản_không_tồn_tại_9999","password":"MậtKhẩuSai_9999","auth_flow":true}</x:v>
       </x:c>
@@ -3097,26 +3090,17 @@
       <x:c r="A18" s="2" t="str">
         <x:v>TC_BND_05</x:v>
       </x:c>
-      <x:c r="B18" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C18" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D18" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E18" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B18" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_BND_05</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="str">
+        <x:v>1. Nhập hai chuỗi Unicode sai, submit; kiểm tra HTML không có ký tự thay thế U+FFFD.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không suy ra hỗ trợ tài khoản Unicode hợp lệ.</x:v>
+      </x:c>
+      <x:c r="E18" s="2" t="str"/>
     </x:row>
     <x:row r="19" ht="108.75" customHeight="1">
       <x:c r="A19" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_SEC_01): Verify password input masking
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1421,21 +1421,14 @@
       <x:c r="N19" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O19" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P19" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q19" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O19" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P19" s="2" t="str">
+        <x:v>1. Kiểm tra type; nhập sample; đọc value.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: type=password; input chứa chính xác chuỗi mẫu. Chỉ kiểm tra DOM, không đánh giá mật mã hoặc nhìn màn hình.</x:v>
+      </x:c>
+      <x:c r="Q19" s="2" t="str"/>
       <x:c r="R19" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3106,26 +3099,17 @@
       <x:c r="A19" s="2" t="str">
         <x:v>TC_SEC_01</x:v>
       </x:c>
-      <x:c r="B19" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C19" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D19" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E19" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B19" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_SEC_01</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="str">
+        <x:v>1. Kiểm tra type; nhập sample; đọc value.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: type=password; input chứa chính xác chuỗi mẫu. Chỉ kiểm tra DOM, không đánh giá mật mã hoặc nhìn màn hình.</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="str"/>
     </x:row>
     <x:row r="20" ht="108.75" customHeight="1">
       <x:c r="A20" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_SEC_02): Reject a SQL tautology payload in the username
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1475,21 +1475,14 @@
       <x:c r="N20" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O20" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P20" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q20" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O20" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P20" s="2" t="str">
+        <x:v>1. Nhập payload vào username, password sai; submit; kiểm tra lỗi chung và mẫu lỗi DB.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có mẫu lỗi DB đã kiểm tra; không kết luận toàn hệ thống không SQLi.</x:v>
+      </x:c>
+      <x:c r="Q20" s="2" t="str"/>
       <x:c r="R20" s="2" t="str">
         <x:v>{"payload":"' OR '1'='1","auth_flow":true}</x:v>
       </x:c>
@@ -3115,26 +3108,17 @@
       <x:c r="A20" s="2" t="str">
         <x:v>TC_SEC_02</x:v>
       </x:c>
-      <x:c r="B20" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C20" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D20" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E20" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B20" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_SEC_02</x:v>
+      </x:c>
+      <x:c r="D20" s="2" t="str">
+        <x:v>1. Nhập payload vào username, password sai; submit; kiểm tra lỗi chung và mẫu lỗi DB.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có mẫu lỗi DB đã kiểm tra; không kết luận toàn hệ thống không SQLi.</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="str"/>
     </x:row>
     <x:row r="21" ht="108.75" customHeight="1">
       <x:c r="A21" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_SEC_03): Reject a SQL comment payload in the username
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1529,21 +1529,14 @@
       <x:c r="N21" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O21" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P21" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q21" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O21" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P21" s="2" t="str">
+        <x:v>1. Nhập payload comment ở username, password sai; submit; kiểm tra lỗi chung và mẫu lỗi DB.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có mẫu lỗi DB đã kiểm tra.</x:v>
+      </x:c>
+      <x:c r="Q21" s="2" t="str"/>
       <x:c r="R21" s="2" t="str">
         <x:v>{"payload":"admin' --","auth_flow":true}</x:v>
       </x:c>
@@ -3124,26 +3117,17 @@
       <x:c r="A21" s="2" t="str">
         <x:v>TC_SEC_03</x:v>
       </x:c>
-      <x:c r="B21" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C21" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D21" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E21" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B21" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_SEC_03</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="str">
+        <x:v>1. Nhập payload comment ở username, password sai; submit; kiểm tra lỗi chung và mẫu lỗi DB.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có mẫu lỗi DB đã kiểm tra.</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="str"/>
     </x:row>
     <x:row r="22" ht="108.75" customHeight="1">
       <x:c r="A22" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_SEC_04): Reject a SQL UNION payload in the username
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1583,21 +1583,14 @@
       <x:c r="N22" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O22" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P22" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q22" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O22" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P22" s="2" t="str">
+        <x:v>1. Nhập UNION sample ở username, password sai; submit; kiểm tra lỗi chung và mẫu lỗi DB.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có mẫu lỗi DB; không kiểm tra data extraction hoặc mọi số cột UNION.</x:v>
+      </x:c>
+      <x:c r="Q22" s="2" t="str"/>
       <x:c r="R22" s="2" t="str">
         <x:v>{"payload":"' UNION SELECT NULL, NULL--","auth_flow":true}</x:v>
       </x:c>
@@ -3133,26 +3126,17 @@
       <x:c r="A22" s="2" t="str">
         <x:v>TC_SEC_04</x:v>
       </x:c>
-      <x:c r="B22" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C22" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D22" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E22" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B22" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_SEC_04</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="str">
+        <x:v>1. Nhập UNION sample ở username, password sai; submit; kiểm tra lỗi chung và mẫu lỗi DB.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có mẫu lỗi DB; không kiểm tra data extraction hoặc mọi số cột UNION.</x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="str"/>
     </x:row>
     <x:row r="23" ht="108.75" customHeight="1">
       <x:c r="A23" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_SEC_05): Reject a SQL tautology payload in the password
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1637,21 +1637,14 @@
       <x:c r="N23" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O23" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P23" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q23" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O23" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P23" s="2" t="str">
+        <x:v>1. Nhập username cấu hình và payload ở password; submit; kiểm tra lỗi chung và mẫu lỗi DB.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có mẫu lỗi DB; không phải time-based/blind SQLi.</x:v>
+      </x:c>
+      <x:c r="Q23" s="2" t="str"/>
       <x:c r="R23" s="2" t="str">
         <x:v>{"payload":"' OR '1'='1","auth_flow":true}</x:v>
       </x:c>
@@ -3142,26 +3135,17 @@
       <x:c r="A23" s="2" t="str">
         <x:v>TC_SEC_05</x:v>
       </x:c>
-      <x:c r="B23" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C23" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D23" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E23" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B23" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C23" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_SEC_05</x:v>
+      </x:c>
+      <x:c r="D23" s="2" t="str">
+        <x:v>1. Nhập username cấu hình và payload ở password; submit; kiểm tra lỗi chung và mẫu lỗi DB.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có mẫu lỗi DB; không phải time-based/blind SQLi.</x:v>
+      </x:c>
+      <x:c r="E23" s="2" t="str"/>
     </x:row>
     <x:row r="24" ht="108.75" customHeight="1">
       <x:c r="A24" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_SEC_06): Reject a quote-based SQL error payload in the username
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1691,21 +1691,14 @@
       <x:c r="N24" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O24" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P24" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q24" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O24" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P24" s="2" t="str">
+        <x:v>1. Submit chuỗi dấu nháy ở username; đọc response HTML.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có regex lỗi SQL/Oracle/MySQL/SQLite/PostgreSQL đã kiểm tra.</x:v>
+      </x:c>
+      <x:c r="Q24" s="2" t="str"/>
       <x:c r="R24" s="2" t="str">
         <x:v>{"payload":"'''''","auth_flow":true}</x:v>
       </x:c>
@@ -3151,26 +3144,17 @@
       <x:c r="A24" s="2" t="str">
         <x:v>TC_SEC_06</x:v>
       </x:c>
-      <x:c r="B24" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C24" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D24" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E24" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B24" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C24" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_SEC_06</x:v>
+      </x:c>
+      <x:c r="D24" s="2" t="str">
+        <x:v>1. Submit chuỗi dấu nháy ở username; đọc response HTML.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có regex lỗi SQL/Oracle/MySQL/SQLite/PostgreSQL đã kiểm tra.</x:v>
+      </x:c>
+      <x:c r="E24" s="2" t="str"/>
     </x:row>
     <x:row r="25" ht="108.75" customHeight="1">
       <x:c r="A25" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_SEC_07): Reject an XSS script payload in the username
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1745,21 +1745,14 @@
       <x:c r="N25" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O25" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P25" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q25" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O25" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P25" s="2" t="str">
+        <x:v>1. Submit payload, theo dõi alert trong timeout; xác nhận lỗi auth; kiểm tra node script chứa marker.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có alert và không có active script chứa marker; chỉ đánh giá mẫu này.</x:v>
+      </x:c>
+      <x:c r="Q25" s="2" t="str"/>
       <x:c r="R25" s="2" t="str">
         <x:v>{"payload":"&lt;script&gt;alert('UTC_XSS_TEST')&lt;/script&gt;","auth_flow":true}</x:v>
       </x:c>
@@ -3160,26 +3153,17 @@
       <x:c r="A25" s="2" t="str">
         <x:v>TC_SEC_07</x:v>
       </x:c>
-      <x:c r="B25" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C25" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D25" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E25" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B25" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C25" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_SEC_07</x:v>
+      </x:c>
+      <x:c r="D25" s="2" t="str">
+        <x:v>1. Submit payload, theo dõi alert trong timeout; xác nhận lỗi auth; kiểm tra node script chứa marker.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có alert và không có active script chứa marker; chỉ đánh giá mẫu này.</x:v>
+      </x:c>
+      <x:c r="E25" s="2" t="str"/>
     </x:row>
     <x:row r="26" ht="108.75" customHeight="1">
       <x:c r="A26" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_SEC_08): Reject an XSS image onerror payload in the username
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1799,21 +1799,14 @@
       <x:c r="N26" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O26" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P26" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q26" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O26" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P26" s="2" t="str">
+        <x:v>1. Submit payload, theo dõi alert; kiểm tra lỗi auth và node event handler chứa marker.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có alert và không có active handler chứa marker; chỉ đánh giá mẫu này.</x:v>
+      </x:c>
+      <x:c r="Q26" s="2" t="str"/>
       <x:c r="R26" s="2" t="str">
         <x:v>{"payload":"&lt;img src=x onerror=alert('UTC_XSS_TEST')&gt;","auth_flow":true}</x:v>
       </x:c>
@@ -3169,26 +3162,17 @@
       <x:c r="A26" s="2" t="str">
         <x:v>TC_SEC_08</x:v>
       </x:c>
-      <x:c r="B26" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C26" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D26" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E26" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B26" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C26" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_SEC_08</x:v>
+      </x:c>
+      <x:c r="D26" s="2" t="str">
+        <x:v>1. Submit payload, theo dõi alert; kiểm tra lỗi auth và node event handler chứa marker.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Hiển thị đúng error_text đã cấu hình; form username/password/nút login vẫn hiển thị. Chỉ đánh giá phản hồi từ chối, không cần login thành công. Không có alert và không có active handler chứa marker; chỉ đánh giá mẫu này.</x:v>
+      </x:c>
+      <x:c r="E26" s="2" t="str"/>
     </x:row>
     <x:row r="27" ht="108.75" customHeight="1">
       <x:c r="A27" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_SEC_09): Submit five invalid attempts for a nonexistent username
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1853,21 +1853,14 @@
       <x:c r="N27" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O27" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P27" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q27" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O27" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P27" s="2" t="str">
+        <x:v>1. Reset form và gửi sai 5 lần, xác nhận từng phản hồi.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Mỗi lần đều có lỗi chung và form login; không chứng nhận lockout hoặc rate limit.</x:v>
+      </x:c>
+      <x:c r="Q27" s="2" t="str"/>
       <x:c r="R27" s="2" t="str">
         <x:v>{"attempts":5,"auth_flow":true}</x:v>
       </x:c>
@@ -3178,26 +3171,17 @@
       <x:c r="A27" s="2" t="str">
         <x:v>TC_SEC_09</x:v>
       </x:c>
-      <x:c r="B27" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C27" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D27" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E27" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B27" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C27" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_SEC_09</x:v>
+      </x:c>
+      <x:c r="D27" s="2" t="str">
+        <x:v>1. Reset form và gửi sai 5 lần, xác nhận từng phản hồi.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Mỗi lần đều có lỗi chung và form login; không chứng nhận lockout hoặc rate limit.</x:v>
+      </x:c>
+      <x:c r="E27" s="2" t="str"/>
     </x:row>
     <x:row r="28" ht="108.75" customHeight="1">
       <x:c r="A28" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_SEC_10): Require HTTPS for rejected authentication
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1907,21 +1907,14 @@
       <x:c r="N28" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O28" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P28" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q28" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O28" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P28" s="2" t="str">
+        <x:v>1. Kiểm tra URL/action HTTPS; capture POST/response thật khi submit sai.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: POST và response auth dùng HTTPS, Chrome báo secure; không đánh giá mọi TLS cipher/version.</x:v>
+      </x:c>
+      <x:c r="Q28" s="2" t="str"/>
       <x:c r="R28" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3187,26 +3180,17 @@
       <x:c r="A28" s="2" t="str">
         <x:v>TC_SEC_10</x:v>
       </x:c>
-      <x:c r="B28" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C28" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D28" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E28" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B28" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C28" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_SEC_10</x:v>
+      </x:c>
+      <x:c r="D28" s="2" t="str">
+        <x:v>1. Kiểm tra URL/action HTTPS; capture POST/response thật khi submit sai.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: POST và response auth dùng HTTPS, Chrome báo secure; không đánh giá mọi TLS cipher/version.</x:v>
+      </x:c>
+      <x:c r="E28" s="2" t="str"/>
     </x:row>
     <x:row r="29" ht="108.75" customHeight="1">
       <x:c r="A29" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_SEC_12): Prevent cross-origin embedding of the login page
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2015,21 +2015,14 @@
       <x:c r="N30" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O30" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P30" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q30" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O30" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P30" s="2" t="str">
+        <x:v>1. Mở fixture khác origin; đọc header response; switch iframe và kiểm tra login form bị chặn.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Có XFO DENY/SAMEORIGIN hoặc CSP frame-ancestors; login form không hoạt động trong iframe.</x:v>
+      </x:c>
+      <x:c r="Q30" s="2" t="str"/>
       <x:c r="R30" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3205,26 +3198,17 @@
       <x:c r="A30" s="2" t="str">
         <x:v>TC_SEC_12</x:v>
       </x:c>
-      <x:c r="B30" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C30" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D30" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E30" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B30" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_SEC_12</x:v>
+      </x:c>
+      <x:c r="D30" s="2" t="str">
+        <x:v>1. Mở fixture khác origin; đọc header response; switch iframe và kiểm tra login form bị chặn.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Có XFO DENY/SAMEORIGIN hoặc CSP frame-ancestors; login form không hoạt động trong iframe.</x:v>
+      </x:c>
+      <x:c r="E30" s="2" t="str"/>
     </x:row>
     <x:row r="31" ht="108.75" customHeight="1">
       <x:c r="A31" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_SEC_11): Require POST and keep passwords out of URLs
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -1961,21 +1961,14 @@
       <x:c r="N29" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O29" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P29" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q29" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O29" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P29" s="2" t="str">
+        <x:v>1. Kiểm tra đúng form POST; submit sai; capture request tới action và URL.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Request tới action dùng POST; URL request/trang không chứa invalid_password.</x:v>
+      </x:c>
+      <x:c r="Q29" s="2" t="str"/>
       <x:c r="R29" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3196,26 +3189,17 @@
       <x:c r="A29" s="2" t="str">
         <x:v>TC_SEC_11</x:v>
       </x:c>
-      <x:c r="B29" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C29" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D29" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E29" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B29" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C29" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_SEC_11</x:v>
+      </x:c>
+      <x:c r="D29" s="2" t="str">
+        <x:v>1. Kiểm tra đúng form POST; submit sai; capture request tới action và URL.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Request tới action dùng POST; URL request/trang không chứa invalid_password.</x:v>
+      </x:c>
+      <x:c r="E29" s="2" t="str"/>
     </x:row>
     <x:row r="30" ht="108.75" customHeight="1">
       <x:c r="A30" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_PERF_02): Measure failed-authentication response latency
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2123,21 +2123,14 @@
       <x:c r="N32" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O32" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P32" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q32" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O32" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P32" s="2" t="str">
+        <x:v>1. Reset form và đo submit-to-error với username không tồn tại 3 lần.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Mọi mẫu nhỏ hơn 2000ms theo ngân sách testcase; không đo login thành công.</x:v>
+      </x:c>
+      <x:c r="Q32" s="2" t="str"/>
       <x:c r="R32" s="2" t="str">
         <x:v>{"samples":3,"limit_ms":2000,"auth_flow":true}</x:v>
       </x:c>
@@ -3223,26 +3216,17 @@
       <x:c r="A32" s="2" t="str">
         <x:v>TC_PERF_02</x:v>
       </x:c>
-      <x:c r="B32" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C32" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D32" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E32" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B32" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_PERF_02</x:v>
+      </x:c>
+      <x:c r="D32" s="2" t="str">
+        <x:v>1. Reset form và đo submit-to-error với username không tồn tại 3 lần.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Mọi mẫu nhỏ hơn 2000ms theo ngân sách testcase; không đo login thành công.</x:v>
+      </x:c>
+      <x:c r="E32" s="2" t="str"/>
     </x:row>
     <x:row r="33" ht="108.75" customHeight="1">
       <x:c r="A33" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_PERF_01): Measure auth page load over three cold-cache samples
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2069,21 +2069,14 @@
       <x:c r="N31" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O31" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P31" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q31" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O31" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P31" s="2" t="str">
+        <x:v>1. Xóa/tắt cache; tải auth; đọc Navigation Timing load 3 lần.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Mỗi mẫu hữu hạn, dương, nhỏ hơn ngưỡng cấu hình. Không đại diện SLA toàn hệ thống.</x:v>
+      </x:c>
+      <x:c r="Q31" s="2" t="str"/>
       <x:c r="R31" s="2" t="str">
         <x:v>{"samples":3,"auth_flow":true}</x:v>
       </x:c>
@@ -3214,26 +3207,17 @@
       <x:c r="A31" s="2" t="str">
         <x:v>TC_PERF_01</x:v>
       </x:c>
-      <x:c r="B31" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C31" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D31" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E31" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B31" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C31" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_PERF_01</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="str">
+        <x:v>1. Xóa/tắt cache; tải auth; đọc Navigation Timing load 3 lần.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Mỗi mẫu hữu hạn, dương, nhỏ hơn ngưỡng cấu hình. Không đại diện SLA toàn hệ thống.</x:v>
+      </x:c>
+      <x:c r="E31" s="2" t="str"/>
     </x:row>
     <x:row r="32" ht="108.75" customHeight="1">
       <x:c r="A32" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_PERF_03): Measure TTFB over three cold-cache samples
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2177,21 +2177,14 @@
       <x:c r="N33" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O33" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P33" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q33" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O33" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P33" s="2" t="str">
+        <x:v>1. Xóa/tắt cache, tải auth, đọc TTFB 3 lần.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Mỗi mẫu hữu hạn, dương, nhỏ hơn ngưỡng cấu hình.</x:v>
+      </x:c>
+      <x:c r="Q33" s="2" t="str"/>
       <x:c r="R33" s="2" t="str">
         <x:v>{"samples":3,"auth_flow":true}</x:v>
       </x:c>
@@ -3232,26 +3225,17 @@
       <x:c r="A33" s="2" t="str">
         <x:v>TC_PERF_03</x:v>
       </x:c>
-      <x:c r="B33" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C33" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D33" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E33" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B33" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C33" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_PERF_03</x:v>
+      </x:c>
+      <x:c r="D33" s="2" t="str">
+        <x:v>1. Xóa/tắt cache, tải auth, đọc TTFB 3 lần.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Mỗi mẫu hữu hạn, dương, nhỏ hơn ngưỡng cấu hình.</x:v>
+      </x:c>
+      <x:c r="E33" s="2" t="str"/>
     </x:row>
     <x:row r="34" ht="108.75" customHeight="1">
       <x:c r="A34" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_PERF_04): Measure cold-cache auth page transfer size
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2231,21 +2231,14 @@
       <x:c r="N34" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O34" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P34" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q34" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O34" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P34" s="2" t="str">
+        <x:v>1. Tắt/xóa cache; tải tới network idle; cộng encodedDataLength.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Tổng bytes quan sát hữu hạn/dương và &lt;3145728 bytes; chỉ cửa sổ tải được quan sát.</x:v>
+      </x:c>
+      <x:c r="Q34" s="2" t="str"/>
       <x:c r="R34" s="2" t="str">
         <x:v>{"limit_bytes":3145728,"auth_flow":true}</x:v>
       </x:c>
@@ -3241,26 +3234,17 @@
       <x:c r="A34" s="2" t="str">
         <x:v>TC_PERF_04</x:v>
       </x:c>
-      <x:c r="B34" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C34" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D34" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E34" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B34" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C34" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_PERF_04</x:v>
+      </x:c>
+      <x:c r="D34" s="2" t="str">
+        <x:v>1. Tắt/xóa cache; tải tới network idle; cộng encodedDataLength.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Tổng bytes quan sát hữu hạn/dương và &lt;3145728 bytes; chỉ cửa sổ tải được quan sát.</x:v>
+      </x:c>
+      <x:c r="E34" s="2" t="str"/>
     </x:row>
     <x:row r="35" ht="108.75" customHeight="1">
       <x:c r="A35" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_PERF_05): Measure the auth page request count
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2285,21 +2285,14 @@
       <x:c r="N35" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O35" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P35" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q35" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O35" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P35" s="2" t="str">
+        <x:v>1. Cold load tới network idle; đếm request document/redirect/assets/XHR.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Số request quan sát &gt;0 và &lt;50; không tính traffic sau cửa sổ quan sát.</x:v>
+      </x:c>
+      <x:c r="Q35" s="2" t="str"/>
       <x:c r="R35" s="2" t="str">
         <x:v>{"limit_requests":50,"auth_flow":true}</x:v>
       </x:c>
@@ -3250,26 +3243,17 @@
       <x:c r="A35" s="2" t="str">
         <x:v>TC_PERF_05</x:v>
       </x:c>
-      <x:c r="B35" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C35" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D35" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E35" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B35" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C35" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_PERF_05</x:v>
+      </x:c>
+      <x:c r="D35" s="2" t="str">
+        <x:v>1. Cold load tới network idle; đếm request document/redirect/assets/XHR.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Số request quan sát &gt;0 và &lt;50; không tính traffic sau cửa sổ quan sát.</x:v>
+      </x:c>
+      <x:c r="E35" s="2" t="str"/>
     </x:row>
     <x:row r="36" ht="108.75" customHeight="1">
       <x:c r="A36" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_PERF_06): Test offline authentication and retry after connectivity returns
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2339,21 +2339,14 @@
       <x:c r="N36" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O36" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P36" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q36" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O36" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P36" s="2" t="str">
+        <x:v>1. Mô phỏng offline; submit sai; capture loadingFailed; khôi phục; tải lại và submit sai.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Có bằng chứng transport failure lúc offline; sau restore auth trả lỗi chung. Không coi WebDriver timeout là app timeout.</x:v>
+      </x:c>
+      <x:c r="Q36" s="2" t="str"/>
       <x:c r="R36" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3259,26 +3252,17 @@
       <x:c r="A36" s="2" t="str">
         <x:v>TC_PERF_06</x:v>
       </x:c>
-      <x:c r="B36" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C36" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D36" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E36" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B36" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C36" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_PERF_06</x:v>
+      </x:c>
+      <x:c r="D36" s="2" t="str">
+        <x:v>1. Mô phỏng offline; submit sai; capture loadingFailed; khôi phục; tải lại và submit sai.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Có bằng chứng transport failure lúc offline; sau restore auth trả lỗi chung. Không coi WebDriver timeout là app timeout.</x:v>
+      </x:c>
+      <x:c r="E36" s="2" t="str"/>
     </x:row>
     <x:row r="37" ht="108.75" customHeight="1">
       <x:c r="A37" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_UI_01): Verify authentication controls are visible and enabled
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2393,21 +2393,14 @@
       <x:c r="N37" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O37" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P37" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q37" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O37" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P37" s="2" t="str">
+        <x:v>1. Kiểm tra các control và title.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Ba control visible/enabled, title không rỗng; không đánh giá thiết kế/logo.</x:v>
+      </x:c>
+      <x:c r="Q37" s="2" t="str"/>
       <x:c r="R37" s="2" t="str">
         <x:v>{"auth_flow":true}</x:v>
       </x:c>
@@ -3268,26 +3261,17 @@
       <x:c r="A37" s="2" t="str">
         <x:v>TC_UI_01</x:v>
       </x:c>
-      <x:c r="B37" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C37" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D37" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E37" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B37" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C37" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_UI_01</x:v>
+      </x:c>
+      <x:c r="D37" s="2" t="str">
+        <x:v>1. Kiểm tra các control và title.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Ba control visible/enabled, title không rỗng; không đánh giá thiết kế/logo.</x:v>
+      </x:c>
+      <x:c r="E37" s="2" t="str"/>
     </x:row>
     <x:row r="38" ht="108.75" customHeight="1">
       <x:c r="A38" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_UI_03): Verify Tab order through the authentication form
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2501,21 +2501,14 @@
       <x:c r="N39" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O39" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P39" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q39" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O39" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P39" s="2" t="str">
+        <x:v>1. Click username, TAB qua từng control; so sánh activeElement.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Focus khớp thứ tự khai báo; nếu DOM có checkbox xen giữa thì testcase có thể Fail và phải đối chiếu yêu cầu.</x:v>
+      </x:c>
+      <x:c r="Q39" s="2" t="str"/>
       <x:c r="R39" s="2" t="str">
         <x:v>{"tab_order":["username","password","login"],"auth_flow":true}</x:v>
       </x:c>
@@ -3286,26 +3279,17 @@
       <x:c r="A39" s="2" t="str">
         <x:v>TC_UI_03</x:v>
       </x:c>
-      <x:c r="B39" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C39" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D39" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E39" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B39" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C39" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_UI_03</x:v>
+      </x:c>
+      <x:c r="D39" s="2" t="str">
+        <x:v>1. Click username, TAB qua từng control; so sánh activeElement.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Focus khớp thứ tự khai báo; nếu DOM có checkbox xen giữa thì testcase có thể Fail và phải đối chiếu yêu cầu.</x:v>
+      </x:c>
+      <x:c r="E39" s="2" t="str"/>
     </x:row>
     <x:row r="40" ht="108.75" customHeight="1">
       <x:c r="A40" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_UI_02): Reject a blank password submitted with Enter
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2447,21 +2447,14 @@
       <x:c r="N38" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O38" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P38" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q38" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O38" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P38" s="2" t="str">
+        <x:v>1. Xác nhận empty-password bằng click; tải lại rồi Enter tại password rỗng.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Native invalid hoặc lỗi auth server; form login còn hiển thị.</x:v>
+      </x:c>
+      <x:c r="Q38" s="2" t="str"/>
       <x:c r="R38" s="2" t="str">
         <x:v>{"auth_flow":true,"error_text":"Bạn chưa nhập mật khẩu"}</x:v>
       </x:c>
@@ -3277,26 +3270,17 @@
       <x:c r="A38" s="2" t="str">
         <x:v>TC_UI_02</x:v>
       </x:c>
-      <x:c r="B38" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C38" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D38" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E38" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B38" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C38" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_UI_02</x:v>
+      </x:c>
+      <x:c r="D38" s="2" t="str">
+        <x:v>1. Xác nhận empty-password bằng click; tải lại rồi Enter tại password rỗng.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Native invalid hoặc lỗi auth server; form login còn hiển thị.</x:v>
+      </x:c>
+      <x:c r="E38" s="2" t="str"/>
     </x:row>
     <x:row r="39" ht="108.75" customHeight="1">
       <x:c r="A39" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_UI_04): Compare generic errors and HTTP status for both invalid username types
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2555,21 +2555,14 @@
       <x:c r="N40" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O40" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P40" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q40" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O40" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P40" s="2" t="str">
+        <x:v>1. Submit hai loại trong phiên mới 3 cặp; so error_text, HTTP status; ghi timing.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Thông báo chung cùng nội dung; HTTP status giống nhau. Timing được ghi, không kết luận không enumeration qua timing.</x:v>
+      </x:c>
+      <x:c r="Q40" s="2" t="str"/>
       <x:c r="R40" s="2" t="str">
         <x:v>{"samples":3,"auth_flow":true}</x:v>
       </x:c>
@@ -3295,26 +3288,17 @@
       <x:c r="A40" s="2" t="str">
         <x:v>TC_UI_04</x:v>
       </x:c>
-      <x:c r="B40" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C40" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D40" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E40" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B40" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C40" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_UI_04</x:v>
+      </x:c>
+      <x:c r="D40" s="2" t="str">
+        <x:v>1. Submit hai loại trong phiên mới 3 cặp; so error_text, HTTP status; ghi timing.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Thông báo chung cùng nội dung; HTTP status giống nhau. Timing được ghi, không kết luận không enumeration qua timing.</x:v>
+      </x:c>
+      <x:c r="E40" s="2" t="str"/>
     </x:row>
     <x:row r="41" ht="108.75" customHeight="1">
       <x:c r="A41" s="2" t="str">

</xml_diff>

<commit_message>
test(TC_UI_05): Verify the authentication form at three viewport sizes
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2609,21 +2609,14 @@
       <x:c r="N41" s="2" t="str">
         <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
       </x:c>
-      <x:c r="O41" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P41" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="Q41" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="O41" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="P41" s="2" t="str">
+        <x:v>1. Thay viewport, tải auth, kiểm tra overflow và hit-test control.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Không horizontal overflow; controls có kích thước, nằm trong viewport, enabled và không bị che.</x:v>
+      </x:c>
+      <x:c r="Q41" s="2" t="str"/>
       <x:c r="R41" s="2" t="str">
         <x:v>{"viewports":[[1920,1080],[1366,768],[375,667]],"auth_flow":true}</x:v>
       </x:c>
@@ -3304,26 +3297,17 @@
       <x:c r="A41" s="2" t="str">
         <x:v>TC_UI_05</x:v>
       </x:c>
-      <x:c r="B41" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Manual</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C41" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D41" s="2" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E41" s="2" t="inlineStr">
-        <x:is>
-          <x:t>Chưa triển khai automation; bổ sung trong commit testcase.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B41" s="2" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="C41" s="2" t="str">
+        <x:v>tests.test_login.TestLogin.test_TC_UI_05</x:v>
+      </x:c>
+      <x:c r="D41" s="2" t="str">
+        <x:v>1. Thay viewport, tải auth, kiểm tra overflow và hit-test control.
+2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Không horizontal overflow; controls có kích thước, nằm trong viewport, enabled và không bị che.</x:v>
+      </x:c>
+      <x:c r="E41" s="2" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
test(TC_UI_03): include email login link in tab order
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testcases" sheetId="1" r:id="R2c4d5b40382b4f6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="R1fd3c41593b6475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testcases" sheetId="1" r:id="R2212215ddf2c4d97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="R4105c66b970948b6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2483,7 +2483,7 @@
         <x:v>Username→password→login theo tab_order</x:v>
       </x:c>
       <x:c r="H39" s="2" t="str">
-        <x:v>Focus khớp thứ tự khai báo; nếu DOM có checkbox xen giữa thì testcase có thể Fail và phải đối chiếu yêu cầu.</x:v>
+        <x:v>TAB focuses username, password, the UTC e-mail login link, then the login button.</x:v>
       </x:c>
       <x:c r="I39" s="2" t="str">
         <x:v>Giữ Chrome cho testcase tiếp theo; dọn trạng thái trước test tiếp theo. Chỉ đóng WebDriver khi suite kết thúc.</x:v>
@@ -2499,7 +2499,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="N39" s="2" t="str">
-        <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
+        <x:v>Observed in Chrome on the UTC login page: username → password → UTC e-mail login link → login button.</x:v>
       </x:c>
       <x:c r="O39" s="2" t="str">
         <x:v>Automated</x:v>
@@ -2510,7 +2510,7 @@
       </x:c>
       <x:c r="Q39" s="2" t="str"/>
       <x:c r="R39" s="2" t="str">
-        <x:v>{"tab_order":["username","password","login"],"auth_flow":true}</x:v>
+        <x:v>{"tab_order":["username","password","email","login"],"auth_flow":true}</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="135" customHeight="1">

</xml_diff>

<commit_message>
test(TC_SEC_12): report anti-framing observations
</commit_message>
<xml_diff>
--- a/testcases/TestCases_VanPhongDienTu_UTC.xlsx
+++ b/testcases/TestCases_VanPhongDienTu_UTC.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testcases" sheetId="1" r:id="R2212215ddf2c4d97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="R4105c66b970948b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testcases" sheetId="1" r:id="R210faef657c14625"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="R53dc1b1b2e3f46c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1984,20 +1984,21 @@
         <x:v>Auth / Browser SEC</x:v>
       </x:c>
       <x:c r="D30" s="2" t="str">
-        <x:v>Chống nhúng trang login khác origin</x:v>
+        <x:v>Observe anti-framing controls on the login page</x:v>
       </x:c>
       <x:c r="E30" s="2" t="str">
-        <x:v>Chrome dùng chung cả suite; cookie/storage/cache/network/viewport đã reset trước test. URL và dữ liệu auth âm đã cấu hình. Không cần login thành công.</x:v>
+        <x:v>Fresh browser context; no authenticated session; open the login page in a cross-origin iframe.</x:v>
       </x:c>
       <x:c r="F30" s="2" t="str">
-        <x:v>1. Mở fixture khác origin; đọc header response; switch iframe và kiểm tra login form bị chặn.
-2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi.</x:v>
+        <x:v>1. Capture X-Frame-Options and CSP frame-ancestors from the login response.
+2. Check whether the login form renders in the cross-origin iframe.
+3. Record the observed protection policy and any security finding.</x:v>
       </x:c>
       <x:c r="G30" s="2" t="str">
         <x:v>Fixture localhost iframe tới URL auth</x:v>
       </x:c>
       <x:c r="H30" s="2" t="str">
-        <x:v>Có XFO DENY/SAMEORIGIN hoặc CSP frame-ancestors; login form không hoạt động trong iframe.</x:v>
+        <x:v>Capture response status and anti-framing headers, and record whether the login form renders in a cross-origin iframe. PASS confirms the observation completed, not policy compliance.</x:v>
       </x:c>
       <x:c r="I30" s="2" t="str">
         <x:v>Giữ Chrome cho testcase tiếp theo; dọn trạng thái trước test tiếp theo. Chỉ đóng WebDriver khi suite kết thúc.</x:v>
@@ -2013,14 +2014,13 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="N30" s="2" t="str">
-        <x:v>Phạm vi theo yêu cầu: auth chưa đăng nhập, dữ liệu âm và kiểm tra mẫu qua browser. Ngân sách performance là tiêu chí của testcase, không tuyên bố chuẩn/SLA UTC.</x:v>
+        <x:v>No approved anti-framing policy was provided. This case is an automated baseline observation; the website owner must review any reported finding.</x:v>
       </x:c>
       <x:c r="O30" s="2" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="P30" s="2" t="str">
-        <x:v>1. Mở fixture khác origin; đọc header response; switch iframe và kiểm tra login form bị chặn.
-2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Có XFO DENY/SAMEORIGIN hoặc CSP frame-ancestors; login form không hoạt động trong iframe.</x:v>
+        <x:v>Capture anti-framing response headers and whether the login form renders in a cross-origin iframe; report any finding.</x:v>
       </x:c>
       <x:c r="Q30" s="2" t="str"/>
       <x:c r="R30" s="2" t="str">
@@ -3128,8 +3128,7 @@
         <x:v>tests.test_login.TestLogin.test_TC_SEC_12</x:v>
       </x:c>
       <x:c r="D30" s="2" t="str">
-        <x:v>1. Mở fixture khác origin; đọc header response; switch iframe và kiểm tra login form bị chặn.
-2. Đối chiếu từng kết quả quan sát với Expected Result; lưu bằng chứng nếu lỗi. Assertion: Có XFO DENY/SAMEORIGIN hoặc CSP frame-ancestors; login form không hoạt động trong iframe.</x:v>
+        <x:v>Capture response policy headers and cross-origin iframe rendering.</x:v>
       </x:c>
       <x:c r="E30" s="2" t="str"/>
     </x:row>

</xml_diff>